<commit_message>
Fix B MAIN capacity labels in printable workbooks
</commit_message>
<xml_diff>
--- a/multclass_double_elimination/(28人)配布印刷・手作業用2classDoubleElimination.xlsx
+++ b/multclass_double_elimination/(28人)配布印刷・手作業用2classDoubleElimination.xlsx
@@ -1484,7 +1484,7 @@
         <is>
           <t>B
 MAIN
-11・12名</t>
+12名</t>
         </is>
       </c>
     </row>
@@ -3325,7 +3325,7 @@
         <is>
           <t>B
 MAIN
-11・12名</t>
+12名</t>
         </is>
       </c>
     </row>

</xml_diff>